<commit_message>
v2 tool head parts
</commit_message>
<xml_diff>
--- a/V2 BETA/RRF/Valkyrie Connection Table.xlsx
+++ b/V2 BETA/RRF/Valkyrie Connection Table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30105"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3837cd5b4a1a02ac/Document Library/GitHub/Project-Valkyrie/V2 BETA/RRF/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3267" documentId="8_{C788BE8B-89FF-47EE-BC54-747C3D562542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3699C84-9A73-4AE3-B60D-115B6B92C5A0}"/>
+  <xr:revisionPtr revIDLastSave="3269" documentId="8_{C788BE8B-89FF-47EE-BC54-747C3D562542}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D5FA5CC-68E0-4B6D-BDAB-0C1755B6C739}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{344B6B93-88E2-4E8A-A19A-9E2625195A37}"/>
+    <workbookView xWindow="28680" yWindow="-45" windowWidth="29040" windowHeight="16440" firstSheet="2" activeTab="2" xr2:uid="{344B6B93-88E2-4E8A-A19A-9E2625195A37}"/>
   </bookViews>
   <sheets>
     <sheet name="DUET 3 6HC" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3249" uniqueCount="710">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3249" uniqueCount="711">
   <si>
     <t>Type</t>
   </si>
@@ -2191,13 +2191,16 @@
   <si>
     <t>rpm</t>
   </si>
+  <si>
+    <t>12V DC</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
   </numFmts>
   <fonts count="15">
     <font>
@@ -2748,7 +2751,7 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3462,9 +3465,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3502,7 +3505,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3608,7 +3611,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3750,7 +3753,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -10748,7 +10751,7 @@
         <v>70</v>
       </c>
       <c r="D81" s="71" t="s">
-        <v>81</v>
+        <v>710</v>
       </c>
       <c r="E81" s="39" t="s">
         <v>78</v>

</xml_diff>